<commit_message>
Added forgot password flow
</commit_message>
<xml_diff>
--- a/src/test/resources/CRM Testcases.xlsx
+++ b/src/test/resources/CRM Testcases.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="20">
   <si>
     <t>Testcase scenario</t>
   </si>
@@ -188,7 +188,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -200,6 +200,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
@@ -571,7 +576,7 @@
       <c r="D2" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="E2" t="s" s="16">
+      <c r="E2" t="s" s="21">
         <v>19</v>
       </c>
     </row>
@@ -586,7 +591,7 @@
       <c r="D3" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="E3" t="s" s="17">
+      <c r="E3" t="s" s="22">
         <v>19</v>
       </c>
     </row>
@@ -600,7 +605,7 @@
       <c r="D4" t="s" s="0">
         <v>8</v>
       </c>
-      <c r="E4" t="s" s="18">
+      <c r="E4" t="s" s="23">
         <v>19</v>
       </c>
     </row>
@@ -617,7 +622,7 @@
       <c r="D5" t="s" s="0">
         <v>16</v>
       </c>
-      <c r="E5" t="s" s="19">
+      <c r="E5" t="s" s="24">
         <v>19</v>
       </c>
     </row>
@@ -634,7 +639,7 @@
       <c r="D6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E6" t="s" s="20">
+      <c r="E6" t="s" s="25">
         <v>19</v>
       </c>
     </row>

</xml_diff>